<commit_message>
Add permanent Pedicure Salons mapping to reconciliation sheet
Maps NetSuite category "105 - Pedicure Salons" to customer #14 in the
ריכוז legend so it's picked up automatically in this and future daily
reports, instead of being excluded as unmapped.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E9QvuhBZminJvrtKVH8YY8
</commit_message>
<xml_diff>
--- a/kirill/outputs/2026-08-23.xlsx
+++ b/kirill/outputs/2026-08-23.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="101">
   <si>
     <t xml:space="preserve">דוח מכירות אוגוסט 2026</t>
   </si>
@@ -291,6 +291,9 @@
     <t xml:space="preserve">200 - ROW : 217 - N3W FOODS USA</t>
   </si>
   <si>
+    <t xml:space="preserve">105 - Pedicure Salons</t>
+  </si>
+  <si>
     <t xml:space="preserve">Source: PPlay1.xlsx (cb1e4106), "PPlay1 of uriel (Reporter)", נוצר 23/08/2026 09:06:03, תקופה 2026/Aug, Month-to-Date. נשלפו 10 שורות קטגוריה שיש להן נתונים עד כה החודש, מתוך 12 הקטגוריות במקרא גיליון Pplay1 (2 הקטגוריות הנותרות — 0צרכנים פרטיים, 0שונות — אין להן עדיין נתונים החודש; תקין ל-MTD, לא נתון חסר). לעומת 20/08, כל 10 הקטגוריות כבר היו קיימות ולא נוספה קטגוריה חדשה — עלייה טבעית בסכומים המצטברים (MTD) בכל השורות. שורת "Customers" בדוח המקור (₪623,805.3) היא שורת סה"כ-אב ואינה שווה לסכום שורות הקטגוריה (₪1,086,318.6) — כפי שהיה גם בדוחות הקודמים, זו שורת מטה-דוח שאינה תואמת אף ערך במקרא ולכן לא יובאה (בבדיקת עקביות: ₪1,086,318.6 פחות "0פארמים" [₪459,359.7, שורת סה"כ-אב פנימית] פחות "זיכויים BE" [-₪3,153.8] = ₪623,805.1 ≈ ₪623,805.3, בהתאם למוסכמת עבודה). שורה נוספת בדוח המקור, "זיכויים BE" (₪-3,153.8), שוב אינה תואמת אף ערך במקרא הקבוע (12 הקטגוריות) — הוחרגה לפי מוסכמת "שם תואם בדיוק למקרא", ולא צורפה לקטגוריית BE הקיימת ללא אישור מפורש. מכר נטו = עמודה B × 0.91 (מקדם קבוע, מאושר ב-kirill.md).</t>
   </si>
   <si>
@@ -300,7 +303,7 @@
     <t xml:space="preserve">הערה</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: report.xls (5232f259), Meditex Group IL, Custom Sales by Customer Summary, 01 August 2026 - 31 August 2026, Month-to-Date, נמסר 23/08/2026. נשלפו 14 שורות הסיכום (קטגוריה) שיש להן מכירות עד כה החודש, מתוך 27 הקטגוריות במקרא "ריכוז" (13 הקטגוריות הנותרות אין להן מכירות עדיין החודש — תקין ל-MTD, לא נתון חסר). לעומת 20/08, אותן 14 קטגוריות בדיוק — עלייה טבעית בסכומים המצטברים (MTD) בכל השורות, ללא קטגוריה חדשה. לא יובאו שורות פירוט חשבוניות/לקוחות-בת מהדוח הגולמי (1,673 שורות בקובץ המקור), לפי מוסכמת עבודה. סה"כ שורת "Total" בדוח הגולמי המלא: ₪1,064,315.18 — סכום 14 שורות הקטגוריה שנשלפו הוא ₪1,063,586.31, פער של ₪728.87. **אנומליה לתשומת לב ראובן**: הפער נובע משורת סיכום נוספת בדוח הגולמי, "Total - 105 - Pedicure Salons" (₪728.87), שהיא קטגוריה שיש לה מכירות בפועל החודש לראשונה אך אינה קיימת כלל באף אחת מ-27 שורות מקרא "ריכוז" (בשונה מ"זיכויים BE"/"Customers" ב-PPLAY1, שהן שורות מטה-דוח מוכרות שהוחרגו במכוון — כאן מדובר בקטגוריית-לקוח אמיתית, "105 - Pedicure Salons", שמתאימה מבחינה עסקית ל"מכוני פדיקור" [לקוח #14] בגיליון סה"כ, אך לגיליון "ריכוז" אין עבורה שורת מיפוי כלל — פער במקרא הקבוע, לא רק "אין מכירות עדיין"). בהתאם למוסכמת "שלוף רק שורות שתואמות בדיוק למקרא", הקטגוריה לא יובאה ולא נכללה בחישוב סה"כ הנוכחי — נדרשת החלטת ראובן/המשתמש האם להוסיף שורת מיפוי קבועה ל"105 - Pedicure Salons" בגיליון ריכוז (מול לקוח #14) לדוחות הבאים.</t>
+    <t xml:space="preserve">Source: report.xls (5232f259), Meditex Group IL, Custom Sales by Customer Summary, 01 August 2026 - 31 August 2026, Month-to-Date, נמסר 23/08/2026. נשלפו 15 שורות הסיכום (קטגוריה) שיש להן מכירות עד כה החודש, מתוך 28 הקטגוריות במקרא "ריכוז" (13 הקטגוריות הנותרות אין להן מכירות עדיין החודש — תקין ל-MTD, לא נתון חסר). לעומת 20/08, 14 קטגוריות ותיקות עם עלייה טבעית בסכומים המצטברים (MTD), פלוס קטגוריה חדשה: "105 - Pedicure Salons" (₪728.87). עודכן 23/08/2026: בעבר קטגוריה זו לא הייתה קיימת כלל במקרא "ריכוז" (פער מיפוי, לא "אין מכירות") — אושר במפורש על ידי המשתמש ב-23/08/2026 להוסיף שורת מיפוי קבועה בגיליון ריכוז (שורה 30) בין "105 - Pedicure Salons" ללקוח #14 (מכוני פדיקור), לכל הדוחות מהיום והלאה. לא יובאו שורות פירוט חשבוניות/לקוחות-בת מהדוח הגולמי (1,673 שורות בקובץ המקור), לפי מוסכמת עבודה. סה"כ שורת "Total" בדוח הגולמי המלא: ₪1,064,315.18 — תואם כעת בדיוק לסכום 15 שורות הקטגוריה שנשלפו (₪1,063,586.31 + ₪728.87 = ₪1,064,315.18), כך שלא נותרה מכירה כלשהי שלא סווגה.</t>
   </si>
   <si>
     <t xml:space="preserve">Customer</t>
@@ -979,7 +982,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A3,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A3,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A3,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A3,ריכוז!$C$3:$C$30)</f>
         <v>299421.55</v>
       </c>
     </row>
@@ -991,7 +994,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A4,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A4,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A4,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A4,ריכוז!$C$3:$C$30)</f>
         <v>364884.156</v>
       </c>
     </row>
@@ -1003,7 +1006,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A5,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A5,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A5,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A5,ריכוז!$C$3:$C$30)</f>
         <v>52758.524</v>
       </c>
     </row>
@@ -1015,7 +1018,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A6,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A6,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A6,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A6,ריכוז!$C$3:$C$30)</f>
         <v>106781.267</v>
       </c>
     </row>
@@ -1027,7 +1030,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A7,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A7,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A7,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A7,ריכוז!$C$3:$C$30)</f>
         <v>194403.8</v>
       </c>
     </row>
@@ -1039,7 +1042,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A8,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A8,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A8,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A8,ריכוז!$C$3:$C$30)</f>
         <v>54340.832</v>
       </c>
     </row>
@@ -1051,7 +1054,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A9,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A9,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A9,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A9,ריכוז!$C$3:$C$30)</f>
         <v>61825.41</v>
       </c>
     </row>
@@ -1063,7 +1066,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A10,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A10,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A10,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A10,ריכוז!$C$3:$C$30)</f>
         <v>5016.88</v>
       </c>
     </row>
@@ -1075,7 +1078,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A11,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A11,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A11,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A11,ריכוז!$C$3:$C$30)</f>
         <v>1368.95</v>
       </c>
     </row>
@@ -1087,8 +1090,8 @@
         <v>11</v>
       </c>
       <c r="C12" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A12,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A12,ריכוז!$C$3:$C$29)</f>
-        <v>0</v>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A12,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A12,ריכוז!$C$3:$C$30)</f>
+        <v>728.87</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1099,7 +1102,7 @@
         <v>12</v>
       </c>
       <c r="C13" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A13,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A13,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A13,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A13,ריכוז!$C$3:$C$30)</f>
         <v>0</v>
       </c>
     </row>
@@ -1111,7 +1114,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A14,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A14,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A14,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A14,ריכוז!$C$3:$C$30)</f>
         <v>0</v>
       </c>
     </row>
@@ -1123,7 +1126,7 @@
         <v>14</v>
       </c>
       <c r="C15" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A15,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A15,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A15,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A15,ריכוז!$C$3:$C$30)</f>
         <v>9278.69</v>
       </c>
     </row>
@@ -1134,7 +1137,7 @@
       </c>
       <c r="C16" s="15" t="n">
         <f aca="false">SUM(C3:C15)</f>
-        <v>1150080.059</v>
+        <v>1150808.929</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1145,7 +1148,7 @@
         <v>16</v>
       </c>
       <c r="C17" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A17,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A17,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A17,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A17,ריכוז!$C$3:$C$30)</f>
         <v>265719.72</v>
       </c>
     </row>
@@ -1157,7 +1160,7 @@
         <v>17</v>
       </c>
       <c r="C18" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A18,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A18,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A18,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A18,ריכוז!$C$3:$C$30)</f>
         <v>537.53</v>
       </c>
     </row>
@@ -1168,7 +1171,7 @@
       </c>
       <c r="C19" s="15" t="n">
         <f aca="false">C18+C17+C16</f>
-        <v>1416337.309</v>
+        <v>1417066.179</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1191,7 +1194,7 @@
         <v>20</v>
       </c>
       <c r="C21" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A21,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A21,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A21,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A21,ריכוז!$C$3:$C$30)</f>
         <v>132101.57</v>
       </c>
     </row>
@@ -1203,7 +1206,7 @@
         <v>21</v>
       </c>
       <c r="C22" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A22,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A22,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A22,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A22,ריכוז!$C$3:$C$30)</f>
         <v>10986.57</v>
       </c>
     </row>
@@ -1215,7 +1218,7 @@
         <v>22</v>
       </c>
       <c r="C23" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A23,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A23,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A23,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A23,ריכוז!$C$3:$C$30)</f>
         <v>0</v>
       </c>
     </row>
@@ -1227,7 +1230,7 @@
         <v>23</v>
       </c>
       <c r="C24" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A24,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A24,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A24,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A24,ריכוז!$C$3:$C$30)</f>
         <v>0</v>
       </c>
     </row>
@@ -1239,7 +1242,7 @@
         <v>24</v>
       </c>
       <c r="C25" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A25,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A25,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A25,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A25,ריכוז!$C$3:$C$30)</f>
         <v>0</v>
       </c>
     </row>
@@ -1251,7 +1254,7 @@
         <v>25</v>
       </c>
       <c r="C26" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A26,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A26,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A26,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A26,ריכוז!$C$3:$C$30)</f>
         <v>0</v>
       </c>
     </row>
@@ -1263,7 +1266,7 @@
         <v>26</v>
       </c>
       <c r="C27" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A27,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A27,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A27,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A27,ריכוז!$C$3:$C$30)</f>
         <v>0</v>
       </c>
     </row>
@@ -1275,7 +1278,7 @@
         <v>27</v>
       </c>
       <c r="C28" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A28,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A28,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A28,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A28,ריכוז!$C$3:$C$30)</f>
         <v>0</v>
       </c>
     </row>
@@ -1287,7 +1290,7 @@
         <v>28</v>
       </c>
       <c r="C29" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A29,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A29,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A29,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A29,ריכוז!$C$3:$C$30)</f>
         <v>30237.69</v>
       </c>
     </row>
@@ -1299,7 +1302,7 @@
         <v>29</v>
       </c>
       <c r="C30" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A30,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A30,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A30,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A30,ריכוז!$C$3:$C$30)</f>
         <v>0</v>
       </c>
     </row>
@@ -1311,7 +1314,7 @@
         <v>30</v>
       </c>
       <c r="C31" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A31,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A31,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A31,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A31,ריכוז!$C$3:$C$30)</f>
         <v>0</v>
       </c>
     </row>
@@ -1323,7 +1326,7 @@
         <v>31</v>
       </c>
       <c r="C32" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A32,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A32,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A32,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A32,ריכוז!$C$3:$C$30)</f>
         <v>0</v>
       </c>
     </row>
@@ -1335,7 +1338,7 @@
         <v>32</v>
       </c>
       <c r="C33" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A33,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A33,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A33,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A33,ריכוז!$C$3:$C$30)</f>
         <v>0</v>
       </c>
     </row>
@@ -1347,7 +1350,7 @@
         <v>33</v>
       </c>
       <c r="C34" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A34,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A34,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A34,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A34,ריכוז!$C$3:$C$30)</f>
         <v>18350.05</v>
       </c>
     </row>
@@ -1359,7 +1362,7 @@
         <v>34</v>
       </c>
       <c r="C35" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A35,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A35,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A35,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A35,ריכוז!$C$3:$C$30)</f>
         <v>26105.72</v>
       </c>
     </row>
@@ -1371,7 +1374,7 @@
         <v>35</v>
       </c>
       <c r="C36" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A36,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A36,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A36,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A36,ריכוז!$C$3:$C$30)</f>
         <v>0</v>
       </c>
     </row>
@@ -1383,7 +1386,7 @@
         <v>36</v>
       </c>
       <c r="C37" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A37,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A37,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A37,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A37,ריכוז!$C$3:$C$30)</f>
         <v>0</v>
       </c>
     </row>
@@ -1395,7 +1398,7 @@
         <v>37</v>
       </c>
       <c r="C38" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A38,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A38,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A38,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A38,ריכוז!$C$3:$C$30)</f>
         <v>0</v>
       </c>
     </row>
@@ -1407,7 +1410,7 @@
         <v>38</v>
       </c>
       <c r="C39" s="9" t="n">
-        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A39,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$29,A39,ריכוז!$C$3:$C$29)</f>
+        <f aca="false">SUMIF(Pplay1!$F$3:$F$14,A39,Pplay1!$H$3:$H$14)+SUMIF(ריכוז!$B$3:$B$30,A39,ריכוז!$C$3:$C$30)</f>
         <v>0</v>
       </c>
     </row>
@@ -1428,7 +1431,7 @@
       </c>
       <c r="C41" s="20" t="n">
         <f aca="false">C40+C19</f>
-        <v>1783411.329</v>
+        <v>1784140.199</v>
       </c>
     </row>
   </sheetData>
@@ -1775,7 +1778,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28.25"/>
@@ -2115,6 +2118,18 @@
       <c r="C29" s="29" t="str">
         <f aca="false">IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A29,NetSuite_מקור!$A:$A,0)),"")</f>
         <v/>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="B30" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="C30" s="29" t="n">
+        <f aca="false">IFERROR(INDEX(NetSuite_מקור!$D:$D,MATCH(A30,NetSuite_מקור!$A:$A,0)),"")</f>
+        <v>728.87</v>
       </c>
     </row>
   </sheetData>
@@ -2144,16 +2159,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C1" s="24" t="s">
         <v>47</v>
       </c>
       <c r="D1" s="24" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2293,7 +2308,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="45"/>
@@ -2302,15 +2317,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="30" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="24" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D2" s="24" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2429,6 +2444,14 @@
       </c>
       <c r="D16" s="1" t="n">
         <v>10986.57</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>728.87</v>
       </c>
     </row>
   </sheetData>
@@ -2457,40 +2480,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="30" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="24" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B2" s="24" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="26" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B3" s="27" t="n">
         <v>53881.35</v>
       </c>
       <c r="C3" s="30" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B4" s="27" t="n">
         <v>-4117.21</v>
       </c>
       <c r="C4" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>